<commit_message>
Tidying Shallap data and updating param files to match earlier changes
</commit_message>
<xml_diff>
--- a/Shallap/Parameters/Options_and_NoVegParams.xlsx
+++ b/Shallap/Parameters/Options_and_NoVegParams.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CFyffe\Dropbox\ISTA\EPIC\Modelling\T_and_C\TC_setups\Shallap\Parameters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\group\pelligrp\Project_folders\MountainWater\Tethys_Chloris\Workflow_dev\Scripts\Cat\TeC_Source_Code\Shallap\Parameters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{333A68C9-06B3-4390-8FD8-37711F0962AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB709D0-57E3-4CC0-86CF-FE366B2FFB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{1C5B3D2E-5EDA-40D4-886E-AB020D607408}"/>
+    <workbookView xWindow="-28920" yWindow="-5475" windowWidth="29040" windowHeight="17520" xr2:uid="{1C5B3D2E-5EDA-40D4-886E-AB020D607408}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="182">
   <si>
     <t>Parameters</t>
   </si>
@@ -324,12 +324,6 @@
     <t>Initial snow albedo. Only used if SNOWALB grid is not given in preprocessing.</t>
   </si>
   <si>
-    <t>ms_max</t>
-  </si>
-  <si>
-    <t>Number of soil layers</t>
-  </si>
-  <si>
     <t xml:space="preserve">rho_g </t>
   </si>
   <si>
@@ -577,6 +571,18 @@
   </si>
   <si>
     <t>Root Parameters</t>
+  </si>
+  <si>
+    <t>OPT_soil_th</t>
+  </si>
+  <si>
+    <t>Option for choosing soil thickness inputs, 1= as % of total thickness (0-100%) or =2 when given in cm.</t>
+  </si>
+  <si>
+    <t>soil_th_max</t>
+  </si>
+  <si>
+    <t>Maximum soil depth [mm], used to create Zs and soil_th when OPT_soil_th==1</t>
   </si>
 </sst>
 </file>
@@ -959,7 +965,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5E79857-BD82-4D37-9CAD-397630C3C251}">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.1796875" customWidth="1"/>
@@ -1272,7 +1278,7 @@
         <v>70</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>30</v>
@@ -1287,7 +1293,7 @@
         <v>47</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1301,7 +1307,7 @@
         <v>70</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>49</v>
@@ -1316,7 +1322,7 @@
         <v>48</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1330,7 +1336,7 @@
         <v>70</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>49</v>
@@ -1345,7 +1351,7 @@
         <v>53</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1397,7 +1403,7 @@
         <v>51</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1423,7 +1429,7 @@
         <v>52</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1512,7 +1518,7 @@
         <v>70</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G21" s="2">
         <v>0.12</v>
@@ -1524,7 +1530,7 @@
         <v>68</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1538,7 +1544,7 @@
         <v>70</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G22" s="2">
         <v>145</v>
@@ -1550,7 +1556,7 @@
         <v>69</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -1578,7 +1584,7 @@
     </row>
     <row r="24" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>34</v>
@@ -1662,7 +1668,7 @@
         <v>70</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>81</v>
@@ -1694,7 +1700,7 @@
         <v>70</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>81</v>
@@ -1723,7 +1729,7 @@
         <v>70</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G29" s="2">
         <v>1.8417100000000001E-4</v>
@@ -1749,7 +1755,7 @@
         <v>70</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G30" s="2">
         <v>-0.65521302800000003</v>
@@ -1775,7 +1781,7 @@
         <v>70</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>81</v>
@@ -1795,7 +1801,7 @@
     </row>
     <row r="32" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>95</v>
+        <v>178</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>50</v>
@@ -1803,109 +1809,115 @@
       <c r="C32" s="3" t="s">
         <v>36</v>
       </c>
+      <c r="D32" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>113</v>
+      </c>
       <c r="F32" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G32" s="3">
+        <v>2</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="G32" s="3">
+      <c r="G33" s="3">
+        <v>2500</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>95</v>
+      </c>
+      <c r="B34" t="s">
+        <v>50</v>
+      </c>
+      <c r="C34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E34" t="s">
+        <v>81</v>
+      </c>
+      <c r="F34" t="s">
+        <v>56</v>
+      </c>
+      <c r="G34">
+        <v>0.35</v>
+      </c>
+      <c r="H34" t="s">
+        <v>39</v>
+      </c>
+      <c r="I34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G35" s="2">
         <v>10</v>
       </c>
-      <c r="H32" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I32" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>97</v>
-      </c>
-      <c r="B33" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" t="s">
-        <v>102</v>
-      </c>
-      <c r="E33" t="s">
-        <v>81</v>
-      </c>
-      <c r="F33" t="s">
-        <v>56</v>
-      </c>
-      <c r="G33">
-        <v>0.35</v>
-      </c>
-      <c r="H33" t="s">
-        <v>39</v>
-      </c>
-      <c r="I33" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
+      <c r="H35" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I35" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G34" s="2">
-        <v>10</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I34" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="G35" s="3">
-        <v>10</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I35" s="3" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>106</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>36</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G36" s="3">
         <v>10</v>
@@ -1914,199 +1926,196 @@
         <v>39</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="37" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>36</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F37" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G37" s="3">
+        <v>10</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I37" s="3" t="s">
         <v>107</v>
-      </c>
-      <c r="G37" s="3">
-        <v>250</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E38" s="4" t="s">
-        <v>115</v>
+      <c r="D38" s="3" t="s">
+        <v>110</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="G38" s="3">
-        <v>2</v>
+        <v>250</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="39" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>171</v>
+        <v>111</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="E39" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G39" s="3">
+        <v>2</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I39" s="3" t="s">
         <v>112</v>
-      </c>
-      <c r="E39" s="4"/>
-      <c r="F39" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="G39" s="3">
-        <v>0.2</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I39" s="3" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="40" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>36</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E40" s="4"/>
       <c r="F40" s="3" t="s">
-        <v>174</v>
+        <v>136</v>
       </c>
       <c r="G40" s="3">
-        <v>10000</v>
+        <v>0.2</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>39</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>116</v>
+        <v>170</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>120</v>
+        <v>36</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>112</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="E41" s="4"/>
       <c r="F41" s="3" t="s">
-        <v>107</v>
+        <v>172</v>
       </c>
       <c r="G41" s="3">
-        <v>5</v>
+        <v>10000</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>39</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>119</v>
+        <v>173</v>
       </c>
     </row>
     <row r="42" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G42" s="3">
+        <v>5</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I42" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B42" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="G42" s="3">
+    </row>
+    <row r="43" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G43" s="3">
         <v>0.1</v>
       </c>
-      <c r="H42" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="G43" s="2">
-        <v>600</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>129</v>
+      <c r="H43" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>34</v>
@@ -2115,27 +2124,27 @@
         <v>40</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F44" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G44" s="2">
+        <v>600</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I44" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="G44" s="2">
-        <v>450</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I44" s="2" t="s">
+      <c r="J44" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="45" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>34</v>
@@ -2144,180 +2153,183 @@
         <v>40</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F45" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G45" s="2">
+        <v>450</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="G45" s="2">
-        <v>10</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I45" s="2" t="s">
-        <v>128</v>
+      <c r="J45" s="2" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="46" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>140</v>
+        <v>40</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>56</v>
+        <v>123</v>
       </c>
       <c r="G46" s="2">
-        <v>0.01</v>
+        <v>10</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="47" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>124</v>
+        <v>56</v>
       </c>
       <c r="G47" s="2">
-        <v>500</v>
+        <v>0.01</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>49</v>
+        <v>122</v>
       </c>
       <c r="G48" s="2">
-        <v>-8</v>
+        <v>500</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="49" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G49" s="2">
+        <v>-8</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I49" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F49" s="2" t="s">
+    </row>
+    <row r="50" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G49" s="2">
+      <c r="D50" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G50" s="2">
         <v>0.45</v>
       </c>
-      <c r="H49" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I49" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E50" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="F50" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G50" s="5">
-        <v>1</v>
-      </c>
-      <c r="H50" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I50" s="5" t="s">
-        <v>178</v>
+      <c r="H50" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="51" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
-        <v>142</v>
+        <v>174</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>34</v>
+        <v>177</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D51" s="5" t="s">
-        <v>112</v>
+      <c r="E51" s="5" t="s">
+        <v>175</v>
       </c>
       <c r="F51" s="5" t="s">
         <v>56</v>
       </c>
       <c r="G51" s="5">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="I51" s="5" t="s">
-        <v>147</v>
+        <v>176</v>
       </c>
     </row>
     <row r="52" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>34</v>
@@ -2326,24 +2338,24 @@
         <v>33</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>148</v>
+        <v>56</v>
       </c>
       <c r="G52" s="5">
-        <v>3.7</v>
+        <v>0.75</v>
       </c>
       <c r="H52" s="5" t="s">
         <v>39</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="53" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>34</v>
@@ -2352,24 +2364,24 @@
         <v>33</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="G53" s="5">
-        <v>0.06</v>
+        <v>3.7</v>
       </c>
       <c r="H53" s="5" t="s">
         <v>39</v>
       </c>
       <c r="I53" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="54" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>34</v>
@@ -2378,24 +2390,24 @@
         <v>33</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="G54" s="5">
-        <v>5.9</v>
+        <v>0.06</v>
       </c>
       <c r="H54" s="5" t="s">
         <v>39</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="55" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>34</v>
@@ -2404,97 +2416,94 @@
         <v>33</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="G55" s="5">
+        <v>5.9</v>
+      </c>
+      <c r="H55" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="G56" s="5">
         <v>2</v>
       </c>
-      <c r="H55" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I55" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G56" s="2">
-        <v>0.13</v>
-      </c>
-      <c r="H56" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I56" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>168</v>
+      <c r="H56" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="57" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G57" s="2">
-        <v>0.94</v>
+        <v>0.13</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="58" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>167</v>
+        <v>56</v>
       </c>
       <c r="G58" s="2">
         <v>0.94</v>
@@ -2503,30 +2512,30 @@
         <v>39</v>
       </c>
       <c r="I58" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="J58" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="J58" s="2" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="59" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>124</v>
+        <v>165</v>
       </c>
       <c r="G59" s="2">
-        <v>1496</v>
+        <v>0.94</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>39</v>
@@ -2535,65 +2544,94 @@
         <v>164</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="60" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>161</v>
+        <v>122</v>
       </c>
       <c r="G60" s="2">
-        <v>948</v>
+        <v>1496</v>
       </c>
       <c r="H60" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="61" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F61" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G61" s="2">
+        <v>948</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G61" s="2">
+      <c r="G62" s="2">
         <v>1.6E-2</v>
       </c>
-      <c r="H61" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I61" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="J61" s="2" t="s">
-        <v>168</v>
+      <c r="H62" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>